<commit_message>
add new sources (yves) and add oil as heat source for industry heat (based on new Eurostat dataset)
</commit_message>
<xml_diff>
--- a/input_data/Parametrization/heat_tech_parametrization.xlsx
+++ b/input_data/Parametrization/heat_tech_parametrization.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="7" min="1" max="1"/>
@@ -709,17 +709,22 @@
           <t>biomass_boiler_industry</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>oil_boiler_industry</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>XX_heat_pump</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>comment</t>
         </is>
@@ -748,15 +753,18 @@
       <c r="F2" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Crystal_Ball</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>similar to existing techs</t>
         </is>
@@ -793,17 +801,22 @@
           <t>inf</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>inf</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Crystal_Ball</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>similar to existing techs</t>
         </is>
@@ -832,15 +845,18 @@
       <c r="F4" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Crystal_Ball</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>similar to existing techs</t>
         </is>
@@ -869,15 +885,18 @@
       <c r="F5" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Crystal_Ball</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>similar to existing techs</t>
         </is>
@@ -914,17 +933,22 @@
           <t>inf</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>inf</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Crystal_Ball</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>similar to existing techs</t>
         </is>
@@ -953,15 +977,18 @@
       <c r="F7" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Crystal_Ball</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>similar to existing techs</t>
         </is>
@@ -990,15 +1017,18 @@
       <c r="F8" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="G8" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>Crystal_Ball</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>Crystal Ball heat_pump has a time-varying max_load.csv (per node/year, ~0.27-0.75). What to do?</t>
         </is>
@@ -1027,15 +1057,18 @@
       <c r="F9" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="G9" s="9" t="n">
+      <c r="G9" t="n">
+        <v>21</v>
+      </c>
+      <c r="H9" s="9" t="n">
         <v>19</v>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Crystal_Ball</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>similar to existing techs</t>
         </is>
@@ -1064,15 +1097,18 @@
       <c r="F10" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Crystal_Ball</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>similar to existing techs</t>
         </is>
@@ -1101,15 +1137,18 @@
       <c r="F11" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>combustion CO2 carried on the fuel CARRIER (natural_gas_industry/biomass), not here. Correct?</t>
         </is>
@@ -1138,15 +1177,18 @@
       <c r="F12" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>Crystal_Ball</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr">
         <is>
           <t>similar to existing techs</t>
         </is>
@@ -1175,15 +1217,18 @@
       <c r="F13" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>Crystal_Ball</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>similar to existing techs</t>
         </is>
@@ -1212,15 +1257,18 @@
       <c r="F14" s="8" t="n">
         <v>11.25235822449202</v>
       </c>
-      <c r="G14" s="9" t="n">
+      <c r="G14" t="n">
+        <v>17.3558850780639</v>
+      </c>
+      <c r="H14" s="9" t="n">
         <v>20.35719959610157</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Crystal_Ball</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>similar to existing techs</t>
         </is>
@@ -1249,15 +1297,18 @@
       <c r="F15" s="8" t="n">
         <v>0.29</v>
       </c>
-      <c r="G15" s="9" t="n">
+      <c r="G15" t="n">
         <v>0.29</v>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H15" s="9" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Crystal_Ball</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>similar to existing techs</t>
         </is>
@@ -1286,15 +1337,18 @@
       <c r="F16" s="8" t="n">
         <v>513.6365981866318</v>
       </c>
-      <c r="G16" s="9" t="n">
+      <c r="G16" t="n">
+        <v>487.186345248536</v>
+      </c>
+      <c r="H16" s="9" t="n">
         <v>930.1261448256167</v>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>Crystal_Ball</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="J16" s="4" t="inlineStr">
         <is>
           <t>similar to existing techs</t>
         </is>
@@ -1331,13 +1385,18 @@
           <t>heat_low_temp_industry</t>
         </is>
       </c>
-      <c r="G17" s="9" t="inlineStr">
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>heat_low_temp_industry</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
         <is>
           <t>heat</t>
         </is>
       </c>
-      <c r="H17" s="4" t="n"/>
       <c r="I17" s="4" t="n"/>
+      <c r="J17" s="4" t="n"/>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -1370,13 +1429,18 @@
           <t>biomass</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>oil</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t>electricity</t>
         </is>
       </c>
-      <c r="H18" s="4" t="n"/>
       <c r="I18" s="4" t="n"/>
+      <c r="J18" s="4" t="n"/>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -1409,13 +1473,18 @@
           <t>heat_low_temp_industry</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>heat_low_temp_industry</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
         <is>
           <t>heat</t>
         </is>
       </c>
-      <c r="H19" s="4" t="n"/>
       <c r="I19" s="4" t="n"/>
+      <c r="J19" s="4" t="n"/>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -1440,15 +1509,18 @@
       <c r="F20" s="8" t="n">
         <v>1.197604790419162</v>
       </c>
-      <c r="G20" s="9" t="n">
+      <c r="G20" t="n">
+        <v>1.005025125628141</v>
+      </c>
+      <c r="H20" s="9" t="n">
         <v>0.3305785123966942</v>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>Crystal_Ball</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="J20" s="4" t="inlineStr">
         <is>
           <t>similar to existing techs</t>
         </is>

</xml_diff>

<commit_message>
add coal and waste boilers for industry heat production
</commit_message>
<xml_diff>
--- a/input_data/Parametrization/heat_tech_parametrization.xlsx
+++ b/input_data/Parametrization/heat_tech_parametrization.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="7" min="1" max="1"/>
@@ -729,6 +729,16 @@
           <t>comment</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>coal_boiler_industry</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>waste_boiler_industry</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -769,6 +779,12 @@
           <t>similar to existing techs</t>
         </is>
       </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -821,6 +837,16 @@
           <t>similar to existing techs</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -861,6 +887,12 @@
           <t>similar to existing techs</t>
         </is>
       </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -901,6 +933,12 @@
           <t>similar to existing techs</t>
         </is>
       </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -953,6 +991,16 @@
           <t>similar to existing techs</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -993,6 +1041,12 @@
           <t>similar to existing techs</t>
         </is>
       </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -1033,6 +1087,12 @@
           <t>Crystal Ball heat_pump has a time-varying max_load.csv (per node/year, ~0.27-0.75). What to do?</t>
         </is>
       </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -1073,6 +1133,12 @@
           <t>similar to existing techs</t>
         </is>
       </c>
+      <c r="K9" t="n">
+        <v>21</v>
+      </c>
+      <c r="L9" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -1113,6 +1179,12 @@
           <t>similar to existing techs</t>
         </is>
       </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -1153,6 +1225,12 @@
           <t>combustion CO2 carried on the fuel CARRIER (natural_gas_industry/biomass), not here. Correct?</t>
         </is>
       </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1193,6 +1271,12 @@
           <t>similar to existing techs</t>
         </is>
       </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1233,6 +1317,12 @@
           <t>similar to existing techs</t>
         </is>
       </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" ht="56" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -1273,6 +1363,12 @@
           <t>similar to existing techs</t>
         </is>
       </c>
+      <c r="K14" t="n">
+        <v>17.3558850780639</v>
+      </c>
+      <c r="L14" t="n">
+        <v>17.3558850780639</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1313,6 +1409,12 @@
           <t>similar to existing techs</t>
         </is>
       </c>
+      <c r="K15" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.29</v>
+      </c>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -1353,6 +1455,12 @@
           <t>similar to existing techs</t>
         </is>
       </c>
+      <c r="K16" t="n">
+        <v>487.186345248536</v>
+      </c>
+      <c r="L16" t="n">
+        <v>487.186345248536</v>
+      </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -1397,6 +1505,16 @@
       </c>
       <c r="I17" s="4" t="n"/>
       <c r="J17" s="4" t="n"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>heat_low_temp_industry</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>heat_low_temp_industry</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -1441,6 +1559,16 @@
       </c>
       <c r="I18" s="4" t="n"/>
       <c r="J18" s="4" t="n"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>hard_coal</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>waste</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -1485,6 +1613,16 @@
       </c>
       <c r="I19" s="4" t="n"/>
       <c r="J19" s="4" t="n"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>heat_low_temp_industry</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>heat_low_temp_industry</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -1524,6 +1662,12 @@
         <is>
           <t>similar to existing techs</t>
         </is>
+      </c>
+      <c r="K20" t="n">
+        <v>1.005025125628141</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1.005025125628141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>